<commit_message>
Invoice OCR field accuracy
</commit_message>
<xml_diff>
--- a/Material_Inward_Changelog.xlsx
+++ b/Material_Inward_Changelog.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1890,6 +1890,126 @@
         </is>
       </c>
     </row>
+    <row r="36" ht="90" customHeight="1">
+      <c r="A36" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>August 4, 2026</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>JATIN</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Invoice OCR field accuracy — Outbound Delivery Number fallback, Material Code line-item field, PAN vs Seller GSTIN cross-check, horizontal/photographed invoice prompt fixes</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Client-requested/reported set of Invoice OCR and Extracted Data improvements, delivered together, all scoped to the Invoice tab/prompt only. (1) Outbound Delivery Number fallback: if no legible Invoice Number is present anywhere on the document but an "Outbound Delivery No"/"Delivery No"/"ODN" label is, that value is now used as invoice_number instead -- strictly a fallback, never preferred over a real, readable Invoice Number. (2) Material Code: client specification that these vendor/buyer item codes are always exactly 8 characters and start with "18", "20", "21", or "23" -- added to the OCR prompt as explicit guidance, and a new Material Code column added to the Invoice tab's Goods Information line-item table (both server-rendered rows and the JS-added-row path), with a live amber highlight (visual only, never blocks Save/Approve) flagging any value that doesn't match that 8-character/prefix shape. (3) PAN vs GSTIN cross-check: since a company's 10-character PAN is structurally embedded inside characters 3-12 of its 15-character GSTIN, the Invoice tab's Company PAN field is now compared against the Seller GSTIN on blur -- a mismatch gets the same red .field-expired highlight used for other hard-validation errors (GSTIN checksum, IRN length), since this is a genuine statutory inconsistency rather than a "worth a second look" case. (4) Horizontal/photographed invoice field-accuracy fixes: client reported specific misreads on a horizontal-layout invoice sample for GSTIN, PO Number, Address, Invoice Number, Invoice Date, PAN, and HSN Code -- the OCR prompt gained targeted notes for each: GSTIN/PAN given exact-length sanity checks (15 and 10 characters respectively, cross-referenceable against each other); addresses explicitly instructed to be read as a joined multi-line block rather than just the first word/line (the reported "address extracts as only 1 word" bug); PO Number extended to also check "Customer PO Ref"; Invoice Number/Date given guidance to read the whole small header box on a landscape layout rather than the first date/number-like text found anywhere on the page; HSN/SAC given a distinguishing note versus Material Code and batch/lot numbers. Per the existing non-destructive correction principle (Change 35), none of this repairs or blanks a value server-side beyond the two additions above -- everything else is prompt guidance plus visual-only client-side highlighting.</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>services/extract.py: _build_prompt('invoice') gained new/extended 'Important field notes' entries: invoice_number (Outbound Delivery Number fallback, FALLBACK ONLY, never preferred over a real Invoice Number), invoice_date (landscape header-box guidance), po_number (added "Customer PO Ref"), buyer_address/seller_address/ship_to_address (new note: read and join ALL lines of the address block, not just the first line/word), buyer_gstin/seller_gstin (new note: always exactly 15 characters, re-examine if not), company_pan (new note: always exactly 10 characters, embedded in Seller GSTIN chars 3-12), hsn_sac (new note: distinguish from Material Code and batch/lot numbers), material_code (extended: always exactly 8 characters, starts with 18/20/21/23).
+templates/tabs/extracted_data.html: Goods Information table gained a Material Code &lt;th&gt;/&lt;td&gt; column (server-rendered rows and addGoodsRow()'s JS template), with new _checkMaterialCodeInput()/_checkAllMaterialCodes() functions (event-delegated on #invGoodsBody, amber .field-mismatch highlight if not 8 characters starting with 18/20/21/23) wired to input events and page load. New err_inv_company_pan inline-error div and _validatePanAgainstGstin() function (red .field-expired highlight if Company PAN doesn't match the PAN embedded in Seller GSTIN characters 3-12), wired to blur on both inv_company_pan and inv_seller_gstin.</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Four related improvements to how the Invoice screen reads and checks data. First, if a delivery has no proper Invoice Number printed anywhere but does show an "Outbound Delivery Number", the system now uses that instead of leaving the field blank -- only as a last resort, never in place of a real Invoice Number that's actually there. Second, the Goods Information table on the Invoice screen now has a Material Code column -- these codes always follow a known pattern (8 characters, starting with 18, 20, 21, or 23), so anything that doesn't fit that pattern gets a soft amber highlight as a nudge to double-check it, without blocking anything. Third, the Company PAN field is now automatically checked against the Seller's GST number, since a company's PAN is technically embedded inside its own GST number -- if the two don't agree, the PAN field turns red, the same way other serious mismatches already do. Fourth, based on a specific problem report about a horizontal-style invoice -- where the address was only capturing a single word, and the GSTIN, PO Number, Invoice Number, Invoice Date, PAN, and HSN Code were all coming out wrong -- the scanning instructions were sharpened for each of those fields individually, especially telling it to read a full multi-line address block instead of stopping after the first word.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="90" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>August 4, 2026</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>JATIN</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Remarks &amp; Comments reworked -- comments now show who posted them individually, Remark is now write-once (permanently locked)</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Client-requested revision to the Remarks &amp; Comments feature from Change 32. Two behavioural changes, both scoped to the same shared panel/tables from Change 32 -- no new database tables. (1) Comments now surface the individual username of whoever posted them, not just their role -- get_comments() (database/remarks_operations.py) rewritten from a DISTINCT ON (role) query that returned only the latest comment per role, to a plain chronological SELECT ... ORDER BY created_at ASC returning every comment ever posted, each including created_by AS username (a column that already existed and was already being written on every insert, just never read back out). The now-unused _ROLE_ORDER/_role_sort_key role-ordering helpers were removed since nothing else in the codebase referenced them (confirmed via a full-codebase search before removing). (2) The Remark itself is now write-once: once a Compliance Officer (or SuperAdmin with edit rights) saves a Remark for a record, it is permanently locked -- POST /api/remarks/&lt;history_id&gt; (app.py) now checks for an existing non-empty remark before accepting a new save and rejects with a 403 if one is already set, regardless of role, including SuperAdmin. The database layer (upsert_remark()) is unchanged and technically still supports overwriting -- the lock is enforced one layer up, at the route, matching this codebase's established convention (also used for goods_delivery_mode and ewb_exemption_reasons from Change 33) that the route layer decides permission/lock rules while the db layer just executes the write. Later reviewers who want to add their own input now use Comments instead, which remain unlimited and append-only as before. No database schema changes were needed for either part -- the username column and the remark/comment tables already existed from Change 32.</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>database/remarks_operations.py: get_comments() rewritten -- SQL changed from SELECT DISTINCT ON (role) ... ORDER BY role, created_at DESC to SELECT role, created_by AS username, comment_text, created_at ... ORDER BY created_at ASC, returning the full chronological history instead of one row per role. Removed the now-unused _ROLE_ORDER list and _role_sort_key() helper. Module docstring updated to describe the new write-once Remark and full-history Comments behaviour.
+app.py: api_get_remarks() -- added username to each comment in the response, and a locked boolean to the remark object (true once a non-empty Remark has ever been saved). api_save_remark() -- added a write-once guard: fetches the existing remark via get_remark() before accepting the request body, returns 403 "Remark already set..." if one already exists with non-empty text, for any role including SuperAdmin.
+templates/tabs/_remarks_panel.html: 'Edit Remark' button (renamed 'Add Remark') now hidden by default and only shown by _renderRemark() when the fetched remark is not yet locked; once locked, the edit box is force-hidden and the button stays hidden permanently, with the remark's meta line noting "-- locked, cannot be edited". _renderComments() now shows each comment's username alongside its role tag (new .remarks-comment-role-tag CSS) instead of the role alone.
+database/schema.sql: Updated the stale comment above the history_comments table definition (previously described the old "latest row per role, role-only" behaviour) to describe the current full-history/username behaviour -- no actual column or table change, just an accuracy fix to match the code above.</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Two changes to the Remarks &amp; Comments panel that's on every tab. First, comments now show the actual name of the person who posted them (with their role shown alongside), instead of just their role -- so it's clear exactly who said what, not just which department. Second, the main Remark -- the one written by the Compliance Officer while reviewing a record -- can now only ever be set once. Once it's saved, there's no more 'Edit Remark' button for anyone, including a SuperAdmin -- it's locked in permanently. If someone reviewing the record later has something to add, they post it as a Comment underneath instead, which still works exactly as before and can be added to at any time by anyone with access. Nothing needed to change in the database itself for either of these -- the information was already being stored, it just wasn't being shown or locked down the right way yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="90" customHeight="1">
+      <c r="A38" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>August 5, 2026</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>JATIN</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Bug fix — Invoice OCR JSON breakage from multi-line addresses, and records silently marked "success" with a missing Invoice tab</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Client-reported: a record (history_id 42) showed as processed but the Invoice tab was not visible to the Compliance Officer. Root cause traced through the application logs to two related issues, one of which was a regression introduced by Change 36 earlier this session. (1) Change 36's OCR prompt told the model it could join a multi-line address block "with commas or line breaks" -- for this invoice's ship_to_address (a genuinely multi-line address), the model inserted a literal, unescaped newline character into the JSON string value instead of a comma. A raw newline inside a JSON string is invalid per the JSON spec, so _parse_response() (services/extract.py) failed to parse the ENTIRE invoice response with "Expecting ',' delimiter", discarding every field, not just the address -- reproduced identically on both the automated first pass and the manual Re-run, confirming it was deterministic, not a transient glitch. (2) Independently of the prompt bug, both places that decide whether OCR "succeeded" (folder_watcher.py._process_batch(), the automated intake path, and app.py.api_rerun_ocr(), the manual Re-run OCR button) considered the record successful as long as ANY document type was extracted, not specifically the Invoice. Since E-Way Bill and LR both extracted fine for this record, the record got marked ocr_status="success" and Gate In/MIGO/MIRO form tables got populated, even though invoice_data was never saved -- so the record looked fully processed everywhere except the one tab that actually mattered. A related pre-existing issue was also fixed while in this code: the original automated batch previously aborted and discarded ALL already-successful extractions the instant any single document type failed (a failed Invoice used to also throw away a perfectly good E-Way Bill read) -- each document type is now attempted and saved independently. Fix has two parts: (A) hardened the OCR prompt/parser -- the prompt now explicitly forbids raw line breaks inside any field value (multi-line fields must be joined with a comma and space only), a new self-verification checklist item reinforces this, and _parse_response() gained a defensive _sanitize_json_control_chars() pass that repairs a stray raw newline/tab found inside a JSON string before parsing, as a safety net in case a future prompt/model slip reintroduces the issue. (B) Invoice is now the sole determinant of OCR success in both places -- folder_watcher.py._process_batch() and app.py.api_rerun_ocr() only mark a record "success" if the Invoice specifically was extracted and saved; if other documents succeed but Invoice does not, those documents are still saved (not discarded) but the record correctly stays "failed" until a Re-run actually recovers the Invoice.</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>services/extract.py: base_instructions gained a new global rule forbidding raw line breaks inside any field value (multi-line fields must be joined with ", " only). The buyer_address/seller_address/ship_to_address field note rewritten to remove "or line breaks" and mandate comma-and-space joining with an explicit example. Self-verification checklist gained item 6 (no field contains an actual line break). New _sanitize_json_control_chars() function -- walks the raw response tracking JSON-string state and replaces a raw newline/carriage-return/tab found INSIDE a string value with a single space, never touching anything outside a string; wired into _parse_response() immediately after markdown-fence stripping, before the first json.loads() attempt.
+services/folder_watcher.py: _process_batch()'s OCR loop no longer breaks on the first failed document type -- each type (invoice/ewaybill/lr) is now attempted independently and tracked in a new failures dict. Extracted data for every type that DID succeed is now saved unconditionally (previously gated behind "all types succeeded"). Overall batch success (ocr_succeeded, which drives the ocr_done/ move + ocr_status="success") is now specifically bool(extracted["invoice"]) instead of "no type failed" -- Invoice is the anchor document, matching the same principle already used for the missing-file case in Change 33. The failure-path error_detail/alert now specifically reports the Invoice failure reason, with any other non-blocking failures logged separately.
+app.py: api_rerun_ocr() now tracks invoice_succeeded separately from files_processed. The record is only marked ocr_status="success" if the Invoice specifically was recovered this retry; if other documents recovered but Invoice didn't, the route now returns a specific error ("Invoice could not be re-extracted ... record remains failed until the Invoice succeeds") instead of the previous behaviour of marking the whole record "success" as long as any file re-extracted.</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>A delivery's paperwork went through the automated scanner, and everything looked normal on the record -- except the Invoice screen itself was empty, because the Invoice specifically had failed to read correctly while the E-Way Bill and Lorry Receipt next to it had succeeded. Two things caused this together. First, an instruction added earlier this session (meant to help the scanner capture full multi-line addresses) accidentally told it it was allowed to use an actual line break when combining address lines -- for one invoice with a real multi-line address, the scanner did exactly that, which technically broke the entire block of information it was sending back, not just the address, so nothing from that invoice got saved at all. That instruction has been corrected to only ever use a comma, and a backup safety check was added so that even if this kind of mistake ever happens again, the system can automatically repair it instead of losing the whole reading. Second, and separately, the system was checking "did anything get read successfully?" instead of "did the Invoice specifically get read successfully?" when deciding whether to mark a delivery as fully processed -- so because the other two documents were fine, it marked the whole thing as done, even though the one document every other screen depends on was missing. That check has been corrected so a delivery is only marked complete once the Invoice itself has actually been captured; if only the other documents come through, the record now correctly stays in a "needs another look" state instead of quietly appearing finished with a blank Invoice screen. Along the way, another related weak spot was also fixed: previously, if only ONE of the three documents failed, the system used to throw away the other two documents' already-successful readings as well -- now each one is kept and saved on its own, regardless of whether the others succeeded.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
robot_scripts: add ZGRN print-to-PDF automation (zgrn.robot + pdf_helper.py); po_fetch diagnostic test case; drop tracked templates.zip, gst_approval: fix spinner incorrectly showing over not run state on tab switch
</commit_message>
<xml_diff>
--- a/Material_Inward_Changelog.xlsx
+++ b/Material_Inward_Changelog.xlsx
@@ -43,7 +43,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -60,6 +60,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F4F8FC"/>
         <bgColor rgb="00F4F8FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4F8FC"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +94,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -116,6 +121,18 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -483,7 +500,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H38"/>
+  <dimension ref="A1:H55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2010,6 +2027,652 @@
         </is>
       </c>
     </row>
+    <row r="39" ht="90" customHeight="1">
+      <c r="A39" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>August 7, 2026</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Remarks &amp; Comments query rewrite, extraction prompt overhaul, MIGO 103 UI/robot rebuild, folder-watcher and LDAP hardening</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>A large production-hardening batch touching extraction, MIGO 103, and remarks together. services/extract.py's OCR prompt gained roughly 250 lines of additional field-level guidance, continuing the accuracy work from earlier changes. templates/tabs/migo_103.html was substantially rebuilt (383 lines) alongside matching rewrites to robot_scripts/migo_103.robot and migo_105.robot and a new migo103_link.robot, tightening how PO line items are matched and posted through SAP GUI. database/remarks_operations.py was refactored (query logic reworked, with the matching template _remarks_panel.html updated) as groundwork ahead of the later write-once Remark change. services/folder_watcher.py and services/ldap_auth.py received hardening passes for production reliability, and services/rf_runner.py gained additional posting-path robustness. A new database/diagnose_supreme_ai_users.sql utility script was added for diagnosing LDAP-synced user rows directly against the database.</t>
+        </is>
+      </c>
+      <c r="F39" s="9" t="n">
+        <v>14</v>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>app.py; database/diagnose_supreme_ai_users.sql (NEW); database/remarks_operations.py; database/schema.sql; robot_scripts/migo103_link.robot, migo_103.robot, migo_105.robot; services/extract.py, folder_watcher.py, ldap_auth.py, rf_runner.py; templates/history.html, tabs/_remarks_panel.html, tabs/extracted_data.html, tabs/migo_103.html</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
+        <is>
+          <t>A broad production-readiness pass covering several areas at once: the document-reading AI got more detailed instructions to improve accuracy, the MIGO 103 (goods receipt) screen and its SAP robot were substantially rebuilt for more reliable PO matching, the Remarks feature's underlying logic was reworked as groundwork for a later change, and the background folder-watching and login systems were hardened for smoother day-to-day production use. A new diagnostic script was also added to help troubleshoot LDAP-synced user accounts directly against the database.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="90" customHeight="1">
+      <c r="A40" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>August 7, 2026</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>MANAS</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>Record Admin feature introduced -- delete/reset/revert with full audit log (v21)</t>
+        </is>
+      </c>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>Introduced the Record Admin capability from scratch: a new database/admin_operations.py module (311 lines) providing delete-record, reset-step, and revert-approval actions, every one of which logs to a new admin_action_log table (schema_migration_v21.sql) before acting, capturing who did what and when. A new standalone templates/admin_records.html page (255 lines) gives a SuperAdmin -- or anyone granted the new record_admin permission, added to templates/user_management.html's role-assignment checkboxes -- a search-driven UI to find a record and apply these actions. Alongside this, robot_scripts/po_fetch.robot and services/gst_runner.py received tuning passes, and services/einvoice_bot.py, taxpayer_search_bot.py, ldap_auth.py and folder_watcher.py got smaller adjustments.</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>15</v>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>app.py; database/admin_operations.py (NEW); database/db_operations.py; database/schema_migration_v21.sql (NEW); robot_scripts/po_fetch.robot; services/einvoice_bot.py, folder_watcher.py, gst_runner.py, ldap_auth.py, taxpayer_search_bot.py; templates/admin_records.html (NEW), history.html, index.html, tabs/migo_103.html, user_management.html</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>Added a brand-new "Record Admin" capability so a SuperAdmin -- or someone specifically given permission -- can delete a record entirely, roll back a step that was done in error, or revert an approval. Every one of these actions is logged with who did it and when, so nothing happens invisibly. A dedicated screen was built for searching up a record and applying these actions safely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="90" customHeight="1">
+      <c r="A41" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>August 7, 2026</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>PO fetch bot: Open Quantity + UOM now captured correctly, MIGO 105 document number and vendor name added (v22)</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>robot_scripts/po_fetch.robot's SAP ME23N scrape was extended to also read each PO line's Open Quantity (SAP's outstanding/undelivered quantity, read off the PO Items grid), persisted via schema_migration_v22.sql's new po_line_items.open_qty column (view-only, informational). Separately, a pre-existing bug was fixed where the robot was already emitting a uom value per line but database/po_operations.py's save function never actually read it into a column -- UOM is now saved correctly. MIGO 105's tab gained its own posted document number display and vendor name, matching the pattern already used on MIGO 103/Gate In.</t>
+        </is>
+      </c>
+      <c r="F41" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>database/po_operations.py; database/schema_migration_v22.sql (NEW); robot_scripts/po_fetch.robot; templates/tabs/documents.html, extracted_data.html, gate_in.html, migo_103.html, migo_105.html, miro.html</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
+        <is>
+          <t>The PO-fetching robot now also pulls in each line's outstanding/undelivered quantity from SAP so reviewers can see at a glance how much of a PO is still open, and a bug where the unit-of-measure was being read but silently thrown away before saving was fixed. The MIGO 105 screen also now shows its own posted document number and the vendor name, matching how the other tabs already work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="90" customHeight="1">
+      <c r="A42" s="10" t="n">
+        <v>42</v>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>August 8, 2026</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>Bug-fix pass across OCR save, Gate In, MIGO 103, and MIRO</t>
+        </is>
+      </c>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>A consolidated bug-fix pass following the previous day's larger MIGO 103/Record Admin/PO-fetch work, touching the OCR save path (database/db_operations.py, services/extract.py), the folder watcher, SAP posting (services/rf_runner.py), and UI corrections across Extracted Data, Gate In, MIGO 103, and MIRO. No new database migration accompanied this pass -- purely corrective, no new features.</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>database/db_operations.py; services/extract.py, folder_watcher.py, rf_runner.py; templates/tabs/extracted_data.html, gate_in.html, migo_103.html, miro.html</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>A cleanup pass fixing a batch of small issues that turned up in the screens and behind-the-scenes automation after the previous day's bigger changes, spanning document scanning, Gate In, MIGO 103, and MIRO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="90" customHeight="1">
+      <c r="A43" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>August 11, 2026</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Record Admin: delete-record and multi-revert actions; Gate In backfill-PO error handling; History page UI bug fixes</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Extended the Record Admin feature with a full delete-record action and the ability to revert multiple approval stages at once (Extracted Data approval and GST approval together, as one combined action), both logged to admin_action_log as before. services/rf_runner.py gained handling for a real-world failure case: a Gate In posted without a PO number, later needing zgatein_update (a separate SAP tcode) run to backfill it -- the automation now recognizes and reports this state clearly instead of failing silently. Several History page display bugs were also fixed. Two commits from this session ("delete record, history page ui bugs, z gatein error handling, multiple revert" and "GST Approval, Extracted Data") touched near-identical file sets and are recorded together here as one logical change.</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>app.py; database/admin_operations.py; services/rf_runner.py; templates/admin_records.html, history.html</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
+        <is>
+          <t>The Record Admin screen can now fully delete a record and revert more than one approval stage at once, both logged the same safe way as before. A specific real-world Gate In problem -- a delivery posted without its PO number, needing a separate SAP step to add it afterward -- is now recognized and reported clearly by the automation instead of just failing. Several small display bugs on the History page were also fixed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="90" customHeight="1">
+      <c r="A44" s="10" t="n">
+        <v>44</v>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>August 11, 2026</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>Dev/production environment path switch (IS_PRODUCTION), PO line item Row Status tracking, Stock Transfer OCR routing</t>
+        </is>
+      </c>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>config/config.py gained an IS_PRODUCTION flag that switches the app's working paths between a production root and a DEV_APP_ROOT default (C:\material_inward), together with a much-expanded .env.template documenting every environment variable this touches. A new database migration was added for PO line item status tracking, read from SAP ME23N's line-deletion indicator icon (get_delflag_status() in sap_helpers.py) so a deleted PO line can be shown greyed-out on MIGO 103 instead of looking identical to an active one. Stock Transfer documents (a distinct OCR-routing path) and several Extracted Data tab fixes were included in the same commit. Note: the migration file that ships this Row Status column is schema_migration_v24.sql, but its own internal header comment still reads "schema_migration_v23.sql -- adds a Row Status column" -- a separate, correctly-named schema_migration_v23.sql already exists for invoice_data.outbound_delivery_number. The filenames on disk are correct and safe to run in order; only the v24 file's internal comment text is stale, flagged here for a future cleanup rather than corrected in this entry.</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>.env.template; .gitignore; SETUP.md; app.py; config/config.py, logger.py; database/db_operations.py, schema.sql, schema_migration_v23.sql (NEW); database/supplier_operations.py; requirements.txt; robot_scripts/dms_excel_writer.py, dms_upload.robot, file_dialog.py</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>The application can now be pointed at either a development environment or the real production one via a single setting, with clearer setup documentation for every configuration option involved. A PO line item that gets deleted in SAP is now shown greyed-out on the MIGO 103 screen instead of looking like a normal, still-valid line. Stock Transfer documents also got their own OCR handling path, and several smaller Extracted Data screen issues were fixed alongside this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="90" customHeight="1">
+      <c r="A45" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>August 12, 2026</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Extraction validation (12-digit EWB, alphanumeric GST/PO/IRN, Delivery Challan fix, date prompt), None-placeholder cleanup, and Others document upload support</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Client-requested validation tightening: E-Way Bill numbers are now validated as exactly 12 digits, and GST/PO/IRN fields are validated as alphanumeric, loosened from stricter prior assumptions that were rejecting legitimate values. A Delivery Challan handling bug was fixed, and the OCR date-extraction prompt was refined. A broader "None"-placeholder cleanup pass (the same class of bug as the July 16 Gate-In fix, this time across additional fields) was completed. Others/unrecognized-document upload support was added to templates/tabs/documents.html -- previously extracted and attached to a record but not actually visible anywhere in the UI, "Others" documents now get their own document card, viewable/downloadable like Invoice/E-Way Bill/LR.</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>app.py; config/config.py; services/extract.py; templates/index.html, tabs/documents.html, tabs/extracted_data.html, tabs/gate_in.html, tabs/migo_103.html</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Several data-quality checks were tightened or corrected: E-Way Bill numbers are now checked for the correct 12-digit length, and GST/PO/IRN numbers accept any valid alphanumeric value instead of being too strict and flagging real values as wrong. A Delivery Challan bug was fixed and date reading was improved. More instances of fields showing the word "None" instead of staying blank were cleaned up. "Other" documents that don't match Invoice/E-Way Bill/LR can now actually be seen and downloaded from the Documents screen, instead of being silently attached with no way to view them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="90" customHeight="1">
+      <c r="A46" s="10" t="n">
+        <v>46</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>August 12, 2026</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>MANAS</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>PO fetch bot rewrite, DMS upload/consolidation improvements, RF queue worker tuning</t>
+        </is>
+      </c>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>A large robot/backend-focused batch: robot_scripts/po_fetch.robot rewritten substantially (421 lines changed) alongside sap_helpers.py gaining new SAP GUI helper functions, continuing the PO-fetch accuracy work from the two Record Admin/PO-fetch changes earlier this week. services/rf_queue_worker.py (the background SAP-posting queue processor) received a tuning pass. DMS (document management system) upload and consolidation (dms_upload.robot, dms_excel_writer.py, doc_consolidator.py, file_dialog.py) were adjusted together. services/extract.py and services/einvoice_bot.py received smaller follow-on fixes.</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>18</v>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>app.py; config/config.py, logger.py; database/db_operations.py, po_operations.py, schema_migration_v22.sql, schema_migration_v24.sql (as first added), supplier_operations.py; robot_scripts/dms_excel_writer.py, dms_upload.robot, file_dialog.py, po_fetch.robot, sap_helpers.py; services/doc_consolidator.py, einvoice_bot.py, extract.py, folder_watcher.py, rf_queue_worker.py</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>A large batch of behind-the-scenes improvements to the SAP-automation robots -- especially the one that fetches Purchase Order details -- along with tuning to the background queue that posts approved records into SAP, and to the document-management (DMS) upload and file-consolidation process that runs after MIGO 103.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="90" customHeight="1">
+      <c r="A47" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>August 13, 2026</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>History page: Pending count, card/dropdown sync, date-only filter (v25); Gate In Vendor Name / Vendor Code split with SAP posting fix</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>History page fixes: the "Pending" dashboard count now correctly matches the table's own Pending filter (both were drifting out of sync before this), the status count cards and the status filter dropdown were made to stay in sync with each other, the date filter was simplified to a single-row, date-only control, and "Clear Filters" now resets to a sensible default. Separately, Gate In's Vendor Name field is now split into two: a free-text Vendor Name and a resolved Vendor Code (gate_in_entries.vendor_code, schema_migration_v25.sql) -- previously the single Vendor Name field got silently overwritten with the raw SAP vendor code once Fetch resolved one, losing the human-readable name. services/rf_runner.py's SAP posting was corrected to send the right one of the two to the right SAP field. Includes a same-day follow-up commit ("left out a migration in commit") that added the migration file omitted from the first commit.</t>
+        </is>
+      </c>
+      <c r="F47" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>app.py; database/db_operations.py, gatein_operations.py, schema.sql, schema_migration_v25.sql (NEW); services/rf_runner.py; templates/history.html, tabs/gate_in.html</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
+        <is>
+          <t>Several History page display bugs were fixed so the record counts, filter dropdown, and status cards all agree with each other and with what the table actually shows, and the date filter was simplified into one clean row. On the Gate In screen, Vendor Name and Vendor Code are now two separate fields instead of one field that used to silently overwrite the readable vendor name with a raw SAP code once looked up -- so both stay visible and correct, and the right one gets posted to the right place in SAP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="90" customHeight="1">
+      <c r="A48" s="10" t="n">
+        <v>48</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>August 13, 2026</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>Extracted Data rebuilt as an Excel-style grid; Category picker (Stores/Sales Return/Job Work, v26); MIGO 103 auto-pair popup and panel-order fixes</t>
+        </is>
+      </c>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>The single largest UI change of this stretch: templates/tabs/extracted_data.html was substantially rebuilt into the Excel-style grid layout (bordered attribute/value table bands) that later changes this session continued to refine. A new history.category field (Stores / Sales Return / Job Work, schema_migration_v26.sql) lets Compliance tag each record, which then auto-fills onto the Gate In form's own category selector, with a confirmation prompt if Gate In tries to change it from what Compliance already chose. The previous per-section Save buttons (Invoice/E-Way Bill/LR each saved separately) were replaced with one shared Save-and-Proceed action. MIGO 103's Auto-Pair popup (which suggests matching a fetched PO line to the invoice) was fixed to stop firing automatically just from loading the page -- it now only triggers on an actual user action -- and the MIGO 103/105 header and detail panels were changed to auto-open before the PO data fills in, rather than after.</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>10</v>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>app.py; database/scenario_operations.py, schema_migration_v26.sql (NEW); robot_scripts/migo_103.robot, migo_105.robot, po_fetch.robot; services/rf_runner.py; templates/tabs/extracted_data.html, gate_in.html, migo_103.html</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>This was the biggest visible redesign of the Extracted Data screen in this stretch -- it moved to a clean, Excel-style grid layout that later work in this session built on top of. A new Category field (Stores, Sales Return, or Job Work) lets the Compliance Officer classify each delivery, and that choice now automatically carries over to the Gate In screen instead of needing to be picked twice, with a warning if someone tries to change it there. Saving extracted data also got simpler -- one Save-and-Proceed button instead of a separate save for each document. On MIGO 103, a popup that suggests matching a PO line was fixed so it no longer pops up just from opening the page, and the layout now opens its panels in a more sensible order while PO data is loading in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="90" customHeight="1">
+      <c r="A49" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>August 13, 2026</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Extracted Data grid: styling pass -- cell colours, spacing, equal-height panels, always-open Remarks (client feedback)</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>A focused visual-polish follow-up to the grid rebuild earlier the same day, entirely CSS/styling: light blue cell fill and light yellow section labels (matching the existing status bar's colour scheme), bolder field caption text, a wider gap between the first and second band of fields, Material Info and Tax Info resized to align 50/50 with the bands above them, E-Way Bill Details and LR Details stretched to equal height so the two side-by-side panels line up evenly, and the Remarks panel changed to always-open (expanded by default) specifically on this tab, without affecting how Remarks behaves on any other tab.</t>
+        </is>
+      </c>
+      <c r="F49" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>templates/tabs/extracted_data.html</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
+        <is>
+          <t>A same-day follow-up purely on appearance -- client feedback after seeing the new grid layout asked for specific colour, spacing, and alignment tweaks, all of which were applied here: matching colours to the rest of the page, clearer bold labels, better spacing between sections, evenly-aligned panels, and the Remarks section left open by default on this tab so it doesn't need an extra click to see.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="90" customHeight="1">
+      <c r="A50" s="10" t="n">
+        <v>50</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>August 14, 2026</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>MANAS</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>"Others" document upload now enforces one file at a time (replaces, doesn't accumulate)</t>
+        </is>
+      </c>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>Fixed a gap in the Others/unrecognized-document handling added on August 12: unlike Invoice/E-Way Bill/LR (each of which upserts a single database row per record and so can never accumulate duplicates), the underlying history_extras table had no such constraint for "Others" uploads -- uploading a replacement Others document via the Documents tab, or having one arrive again through automated intake, just added another row alongside the old one instead of replacing it. New database/scenario_operations.py function delete_history_extras_by_doctype() now runs before every Others upload, removing any existing Others row(s) for that record (and returning their filenames so app.py can also delete the now-orphaned files from disk) -- enforcing "at most one Others document per record" the same way the other three document types already behave implicitly. Deliberately does not touch genuinely unrecognized/misnamed files (doc_type='extra'), where more than one attaching to the same record is normal, not a duplicate.</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>app.py; database/scenario_operations.py; services/folder_watcher.py</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>Fixed a small gap from the recent "Others" document feature: uploading a replacement Other document used to just pile it up alongside the old one instead of swapping it out, unlike Invoice, E-Way Bill, and LR, which have always correctly replaced their old version. Now, uploading a new Others document correctly replaces the previous one, including cleaning up the old file so it doesn't linger unused.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="90" customHeight="1">
+      <c r="A51" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>August 14, 2026</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Extracted Data: Invoice/Transport bands rebuilt into strict 2-cell Attribute|Value rows; top banner consolidated; Tax Info trimmed; Material Info source badge</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Follow-on refinement to the Excel-grid rebuild, per a client hand-sketch: every Invoice Data and Transport Details band (Doc details, Buyer/Seller/Shipping info, E-Way Bill Details, LR Details) was rebuilt into a strict, consistent "Attribute Name | Value" two-cell row format, replacing an earlier caption-above-input layout. Bill To State and Bill To Code were merged into one "CODE - STATE" display field (same pattern applied to Ship To State), Seller Company PAN was relabeled for clarity, Tax Info was trimmed down to 5 read-only fields, and a "Based on Invoice" source badge was added to the Material Info card so it's clear which document a line item's data originated from. The various top-of-tab status banners were consolidated into one row.</t>
+        </is>
+      </c>
+      <c r="F51" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>app.py; templates/tabs/extracted_data.html</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
+        <is>
+          <t>Continued refining the grid layout from a client sketch: every field on the Invoice and Transport screens now consistently shows its label and value side-by-side in the same clean two-column style throughout, rather than mixing formats. Bill To State/Code and Ship To State/Code were combined into a single, more compact field each. Tax Info was trimmed to just the essentials, and a small badge now shows that the Material Info table's data comes from the Invoice specifically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="90" customHeight="1">
+      <c r="A52" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>August 14, 2026</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>GST Verification made fully on-demand (all auto-triggers removed) with a new admin page; fixed address-blank bug, approval banner, and GDM/EWB picker data-loss</t>
+        </is>
+      </c>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>Client-requested redesign of GST Verification from an automatic, always-running background check into a fully on-demand action. Removed all 4 remaining call sites that silently started the GST bot (on invoice save, on GSTIN edit, on OCR re-run, and on merely opening the GST Approval tab to poll status) -- api_gst_status is now strictly read-only. Added POST /api/gst/run/&lt;id&gt; (first-time trigger) and POST /api/gst/bulk_run (accepts a list of history_ids, used by both the single Re-run button and the new admin page's multi-select), replacing the old two-button (Refresh/Re-run) layout on the GST Approval tab with one button whose label/action changes based on state (Run / Checking... / Re-run). Built a new standalone GST Verification admin page (lists every GST-eligible record with its status, supports search, and bulk-runs selected records) and a matching nav link, gated to Compliance/SuperAdmin. Separately fixed a long-standing bug where Buyer/Seller/Ship-To addresses rendered with zero height (and therefore looked blank) the first time the Extracted Data tab was viewed after page load -- root-caused to the address auto-grow script running while the tab's container was still display:none (so scrollHeight read 0) -- fixed with a MutationObserver that reruns the height calculation once the tab actually becomes visible. Also fixed: the Approved-By banner's wording was simplified, the Category/Goods Delivery Mode/E-Way Bill Exemption banners were split into independent boxes shown only when applicable, and picking a Goods Delivery Mode or E-Way Bill Exemption reason after already editing other Extracted Data fields no longer wipes those in-progress edits with a full page reload.</t>
+        </is>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G52" s="11" t="inlineStr">
+        <is>
+          <t>app.py; database/gst_operations.py; templates/tabs/extracted_data.html, gate_in.html, gst_approval.html; templates/gst_verification_admin.html (NEW); templates/index.html</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="inlineStr">
+        <is>
+          <t>GST Verification no longer runs automatically in the background at all -- it only starts when someone deliberately clicks a button, either for one record from its own GST Approval tab or for a batch of records at once from a new dedicated GST Verification admin page built for Compliance to work through their queue. Separately, a real bug was fixed where a buyer's or seller's address would sometimes appear completely blank the first time a record's Extracted Data tab was opened, even though the address had actually been read correctly -- it was a rendering timing issue, not a data problem. A few smaller polish items were also addressed: the "Approved" banner's wording was simplified, the Category/Delivery Mode/Exemption status boxes now only show up when relevant, and choosing a delivery mode or exemption reason no longer wipes out other in-progress edits on the page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="90" customHeight="1">
+      <c r="A53" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>August 14, 2026</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Removed duplicate GDM/E-Way Bill status box, dropped Extras panel, added highlight styling to "View Original" document links</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>The Goods Delivery Mode / E-Way Bill Exemption "locked" confirmation box was rendering twice -- once in the top status banner row and again as a separate full-width box further down the page -- the redundant lower box was removed entirely once a value is set; the picker itself still appears in its original spot only while a choice is still needed. The "Extras -- N unrecognized files from intake" panel was removed from the Extracted Data tab per client request. "View original invoice" / "View original E-Way Bill" / "View original LR" links were restyled as bordered highlight chips instead of plain text, making them easier to spot.</t>
+        </is>
+      </c>
+      <c r="F53" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>templates/tabs/extracted_data.html</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
+        <is>
+          <t>A quick cleanup: the same "Delivery Mode confirmed" / "Exemption reason confirmed" message was showing up twice on the page, so the duplicate was removed. A panel listing unrecognized extra files was removed from this screen since it wasn't needed there. And the links to view the original scanned documents now stand out as clear highlighted buttons instead of blending in as plain text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="90" customHeight="1">
+      <c r="A54" s="10" t="n">
+        <v>54</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>August 14, 2026</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>Gate In fully decoupled from GST Verification; Invoice Data column alignment fixed; admin pages cross-linked; History filter/status corrected; new GST Verified column</t>
+        </is>
+      </c>
+      <c r="E54" s="11" t="inlineStr">
+        <is>
+          <t>The last remaining hard dependency between GST Verification and the rest of the workflow was removed: Gate In now unlocks purely on Extracted Data approval (app.py's _check_step_allowed and _extracted_data_view_state no longer check history.gst_check at all), so GST Verification can be run before, during, long after, or never in relation to Gate In, with zero effect on whether Gate In can be posted. The Gate In banner was simplified to match. Fixed a real, client-reported knock-on bug this decoupling exposed: the History page's "Data Approved" filter/status was defined as approved-AND-GST-not-yet-checked, so a record that got GST-checked before Gate In happened would silently disappear from the "Data Approved" queue a Gate In user was working from -- corrected so the bucket is purely approval_status-based. "GST Approved" was removed as a pipeline stage/status badge entirely, replaced with a dedicated, Compliance/SuperAdmin-only "GST Verified" Yes/No column, and "Gate In Done" was relabeled "Gate In Approved" for consistency. Separately: fixed inconsistent column alignment across the Invoice Data grid's 6 boxes (each was sizing its label column to its own longest label rather than a shared fixed width) by giving every label column the same fixed width. The four separate, differently-built admin page headers (History, User Management, Record Admin, GST Verification) were unified so each links to all the others, and User Management gained a visible "Back to History" link it was missing. GST Verification's own admin page gained a Not Run / Approved / All status filter (default Not Run) and pagination reduced to 20 rows.</t>
+        </is>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>app.py; database/db_operations.py; templates/admin_records.html, gst_verification_admin.html, history.html, user_management.html; templates/tabs/extracted_data.html, gate_in.html</t>
+        </is>
+      </c>
+      <c r="H54" s="11" t="inlineStr">
+        <is>
+          <t>GST Verification is now completely independent of Gate In in every respect -- Gate In only ever waits on Extracted Data being approved. Fixing this exposed a related bug on the History page, where a record could silently vanish from the "ready for Gate In" list the moment someone happened to run GST Verification on it, even though it was still perfectly ready -- that's now fixed, and GST's own status is shown as its own clearly separate "GST Verified" Yes/No column instead of being mixed into the main progress status. Also in this change: values in the Invoice Data section now line up neatly in a straight column across every box, the History, User Management, Record Admin, and GST Verification screens can all now navigate directly to each other, and the GST Verification admin page got a status filter defaulting to showing only records that still need attention, with a shorter, easier-to-scan page size.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="90" customHeight="1">
+      <c r="A55" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>August 14, 2026</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>MANAS/JATIN</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Added "Copy from Invoice" / "Copy from E-Way Bill" quick-fill buttons on 5 duplicated fields</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Client-requested quick-fill buttons next to 5 fields that duplicate a value already captured elsewhere on the same record, so a reviewer no longer has to retype it by hand: E-Way Bill Details' Inv. No. and Inv. Date copy from Invoice Data's Invoice No./Invoice Date; LR Details' From Location and To Location copy from Invoice Data's Bill To State/Ship To State; LR Details' Vehicle No. copies from E-Way Bill Details' Vehicle No. Each button is a silent overwrite by explicit client decision -- no confirmation prompt even if the target field already has a value -- shows a toast instead if the source field is empty, and is disabled once the record is approved, matching the fields themselves.</t>
+        </is>
+      </c>
+      <c r="F55" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>templates/tabs/extracted_data.html</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>Added small "Copy from Invoice" and "Copy from E-Way Bill" buttons next to 5 fields where the same piece of information is expected to appear on more than one document -- one click fills the field from the other document instead of retyping it by hand. Clicking always overwrites whatever was there before, by design, so it's a fast fix if a value needs correcting too.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>